<commit_message>
edited teams and titles
</commit_message>
<xml_diff>
--- a/ADET/teams and titles of adet.xlsx
+++ b/ADET/teams and titles of adet.xlsx
@@ -728,7 +728,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -736,11 +736,26 @@
       <bottom style="none"/>
       <diagonal style="none"/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal style="none"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -763,11 +778,14 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3191,827 +3209,911 @@
   <cols>
     <col min="1" max="1" style="4" width="9.140625"/>
     <col customWidth="1" min="2" max="2" width="35.7109375"/>
-    <col customWidth="1" min="3" max="3" style="1" width="39.28125"/>
+    <col customWidth="1" min="3" max="3" style="1" width="8.421875"/>
     <col customWidth="1" min="4" max="4" style="3" width="46.421875"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="11" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="2" ht="14.25">
-      <c r="A2" s="4">
+      <c r="A2" s="8">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D2" s="3" t="s">
+      <c r="C2" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D2" s="11" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="3" ht="14.25">
-      <c r="A3" s="4"/>
-      <c r="B3" t="s">
+      <c r="A3" s="8"/>
+      <c r="B3" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="D3" s="3"/>
+      <c r="C3" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="D3" s="11"/>
     </row>
     <row r="4" ht="14.25">
-      <c r="A4" s="4"/>
-      <c r="B4" t="s">
+      <c r="A4" s="8"/>
+      <c r="B4" s="9" t="s">
         <v>167</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D4" s="3"/>
+      <c r="C4" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D4" s="11"/>
     </row>
     <row r="5" ht="14.25">
-      <c r="A5" s="4"/>
-      <c r="B5" t="s">
+      <c r="A5" s="8"/>
+      <c r="B5" s="9" t="s">
         <v>168</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="D5" s="3"/>
+      <c r="C5" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="D5" s="11"/>
     </row>
     <row r="6" ht="14.25">
-      <c r="A6" s="4">
+      <c r="A6" s="8">
         <v>2</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="9" t="s">
         <v>169</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="D6" s="3" t="s">
+      <c r="C6" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="D6" s="11" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="7" ht="14.25">
-      <c r="A7" s="4"/>
-      <c r="B7" t="s">
+      <c r="A7" s="8"/>
+      <c r="B7" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="D7" s="3"/>
+      <c r="C7" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="D7" s="11"/>
     </row>
     <row r="8" ht="14.25">
-      <c r="A8" s="4"/>
-      <c r="B8" t="s">
+      <c r="A8" s="8"/>
+      <c r="B8" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D8" s="3"/>
+      <c r="C8" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D8" s="11"/>
     </row>
     <row r="9" ht="14.25">
-      <c r="A9" s="4"/>
-      <c r="B9" t="s">
+      <c r="A9" s="8"/>
+      <c r="B9" s="9" t="s">
         <v>173</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D9" s="3"/>
+      <c r="C9" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D9" s="11"/>
     </row>
     <row r="10" ht="14.25">
-      <c r="A10" s="4">
+      <c r="A10" s="8">
         <v>3</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D10" s="3" t="s">
+      <c r="C10" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D10" s="11" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="11" ht="14.25">
-      <c r="A11" s="4"/>
-      <c r="B11" t="s">
+      <c r="A11" s="8"/>
+      <c r="B11" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="C11" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D11" s="3"/>
+      <c r="C11" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D11" s="11"/>
     </row>
     <row r="12" ht="14.25">
-      <c r="A12" s="4"/>
-      <c r="B12" s="8" t="s">
+      <c r="A12" s="8"/>
+      <c r="B12" s="9" t="s">
         <v>176</v>
       </c>
-      <c r="C12" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D12" s="3"/>
+      <c r="C12" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D12" s="11"/>
     </row>
     <row r="13" ht="14.25">
-      <c r="A13" s="4"/>
-      <c r="B13" t="s">
+      <c r="A13" s="8"/>
+      <c r="B13" s="9" t="s">
         <v>177</v>
       </c>
-      <c r="C13" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D13" s="3"/>
+      <c r="C13" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D13" s="11"/>
     </row>
     <row r="14" ht="14.25">
-      <c r="A14" s="4">
+      <c r="A14" s="8">
         <v>4</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="C14" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D14" s="3" t="s">
+      <c r="C14" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D14" s="11" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="15" ht="14.25">
-      <c r="A15" s="4"/>
-      <c r="B15" t="s">
+      <c r="A15" s="8"/>
+      <c r="B15" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="C15" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D15" s="3"/>
+      <c r="C15" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D15" s="11"/>
     </row>
     <row r="16" ht="14.25">
-      <c r="A16" s="4"/>
-      <c r="B16" t="s">
+      <c r="A16" s="8"/>
+      <c r="B16" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="C16" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D16" s="3"/>
+      <c r="C16" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D16" s="11"/>
     </row>
     <row r="17" ht="14.25">
-      <c r="A17" s="4"/>
-      <c r="B17" t="s">
+      <c r="A17" s="8"/>
+      <c r="B17" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="C17" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D17" s="3"/>
+      <c r="C17" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D17" s="11"/>
     </row>
     <row r="18" ht="14.25">
-      <c r="A18" s="4">
+      <c r="A18" s="8">
         <v>5</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="9" t="s">
         <v>183</v>
       </c>
-      <c r="C18" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D18" s="3" t="s">
+      <c r="C18" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D18" s="11" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="19" ht="14.25">
-      <c r="A19" s="4"/>
-      <c r="B19" t="s">
+      <c r="A19" s="8"/>
+      <c r="B19" s="9" t="s">
         <v>185</v>
       </c>
-      <c r="C19" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D19" s="3"/>
+      <c r="C19" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D19" s="11"/>
     </row>
     <row r="20" ht="14.25">
-      <c r="A20" s="4"/>
-      <c r="B20" t="s">
+      <c r="A20" s="8"/>
+      <c r="B20" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="C20" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D20" s="3"/>
+      <c r="C20" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D20" s="11"/>
     </row>
     <row r="21" ht="14.25">
-      <c r="A21" s="4"/>
-      <c r="B21" t="s">
+      <c r="A21" s="8"/>
+      <c r="B21" s="9" t="s">
         <v>187</v>
       </c>
-      <c r="C21" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D21" s="3"/>
+      <c r="C21" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D21" s="11"/>
     </row>
     <row r="22" ht="14.25">
-      <c r="A22" s="4">
+      <c r="A22" s="8">
         <v>6</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="9" t="s">
         <v>188</v>
       </c>
-      <c r="C22" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D22" s="3" t="s">
+      <c r="C22" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D22" s="11" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="23" ht="14.25">
-      <c r="A23" s="4"/>
-      <c r="B23" t="s">
+      <c r="A23" s="8"/>
+      <c r="B23" s="9" t="s">
         <v>190</v>
       </c>
-      <c r="C23" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D23" s="3"/>
+      <c r="C23" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D23" s="11"/>
     </row>
     <row r="24" ht="14.25">
-      <c r="A24" s="4"/>
-      <c r="B24" t="s">
+      <c r="A24" s="8"/>
+      <c r="B24" s="9" t="s">
         <v>191</v>
       </c>
-      <c r="C24" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D24" s="3"/>
+      <c r="C24" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D24" s="11"/>
     </row>
     <row r="25" ht="14.25">
-      <c r="A25" s="4"/>
-      <c r="B25" t="s">
+      <c r="A25" s="8"/>
+      <c r="B25" s="9" t="s">
         <v>192</v>
       </c>
-      <c r="C25" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D25" s="3"/>
+      <c r="C25" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D25" s="11"/>
     </row>
     <row r="26" ht="14.25">
-      <c r="A26" s="4">
+      <c r="A26" s="8">
         <v>7</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="9" t="s">
         <v>193</v>
       </c>
-      <c r="C26" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D26" s="3" t="s">
+      <c r="C26" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D26" s="11" t="s">
         <v>194</v>
       </c>
     </row>
     <row r="27" ht="14.25">
-      <c r="A27" s="4"/>
-      <c r="B27" t="s">
+      <c r="A27" s="8"/>
+      <c r="B27" s="9" t="s">
         <v>195</v>
       </c>
-      <c r="C27" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D27" s="3"/>
+      <c r="C27" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D27" s="11"/>
     </row>
     <row r="28" ht="14.25">
-      <c r="A28" s="4"/>
-      <c r="B28" t="s">
+      <c r="A28" s="8"/>
+      <c r="B28" s="9" t="s">
         <v>196</v>
       </c>
-      <c r="C28" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="D28" s="3"/>
+      <c r="C28" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="D28" s="11"/>
     </row>
     <row r="29" ht="14.25">
-      <c r="A29" s="4"/>
-      <c r="B29" t="s">
+      <c r="A29" s="8"/>
+      <c r="B29" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="C29" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="D29" s="3"/>
+      <c r="C29" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="D29" s="11"/>
     </row>
     <row r="30" ht="14.25">
-      <c r="A30" s="4">
+      <c r="A30" s="8">
         <v>8</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="9" t="s">
         <v>198</v>
       </c>
-      <c r="C30" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="D30" s="3" t="s">
+      <c r="C30" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="D30" s="11" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="31" ht="14.25">
-      <c r="A31" s="4"/>
-      <c r="B31" t="s">
+      <c r="A31" s="8"/>
+      <c r="B31" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="C31" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D31" s="3"/>
+      <c r="C31" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D31" s="11"/>
     </row>
     <row r="32" ht="14.25">
-      <c r="A32" s="4"/>
-      <c r="B32" t="s">
+      <c r="A32" s="8"/>
+      <c r="B32" s="9" t="s">
         <v>201</v>
       </c>
-      <c r="C32" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D32" s="3"/>
+      <c r="C32" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D32" s="11"/>
     </row>
     <row r="33" ht="14.25">
-      <c r="A33" s="4"/>
-      <c r="B33" t="s">
+      <c r="A33" s="8"/>
+      <c r="B33" s="9" t="s">
         <v>202</v>
       </c>
-      <c r="C33" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D33" s="3"/>
+      <c r="C33" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D33" s="11"/>
     </row>
     <row r="34" ht="14.25">
-      <c r="A34" s="4">
+      <c r="A34" s="8">
         <v>9</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="9" t="s">
         <v>203</v>
       </c>
-      <c r="C34" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D34" s="3" t="s">
+      <c r="C34" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D34" s="11" t="s">
         <v>204</v>
       </c>
     </row>
     <row r="35" ht="14.25">
-      <c r="A35" s="4"/>
-      <c r="B35" t="s">
+      <c r="A35" s="8"/>
+      <c r="B35" s="9" t="s">
         <v>205</v>
       </c>
-      <c r="C35" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D35" s="3"/>
+      <c r="C35" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D35" s="11"/>
     </row>
     <row r="36" ht="14.25">
-      <c r="A36" s="4"/>
-      <c r="B36" t="s">
+      <c r="A36" s="8"/>
+      <c r="B36" s="9" t="s">
         <v>206</v>
       </c>
-      <c r="C36" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D36" s="3"/>
+      <c r="C36" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D36" s="11"/>
     </row>
     <row r="37" ht="14.25">
-      <c r="A37" s="4"/>
-      <c r="B37" t="s">
+      <c r="A37" s="8"/>
+      <c r="B37" s="9" t="s">
         <v>207</v>
       </c>
-      <c r="C37" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D37" s="3"/>
+      <c r="C37" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D37" s="11"/>
     </row>
     <row r="38" ht="14.25">
-      <c r="A38" s="4">
+      <c r="A38" s="8">
         <v>10</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B38" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="C38" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D38" s="3" t="s">
+      <c r="C38" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D38" s="11" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="39" ht="14.25">
-      <c r="A39" s="4"/>
-      <c r="B39" t="s">
+      <c r="A39" s="8"/>
+      <c r="B39" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="C39" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D39" s="3"/>
+      <c r="C39" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D39" s="11"/>
     </row>
     <row r="40" ht="14.25">
-      <c r="A40" s="4"/>
-      <c r="B40" t="s">
+      <c r="A40" s="8"/>
+      <c r="B40" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="C40" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D40" s="3"/>
+      <c r="C40" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D40" s="11"/>
     </row>
     <row r="41" ht="14.25">
-      <c r="A41" s="4"/>
-      <c r="B41" t="s">
+      <c r="A41" s="8"/>
+      <c r="B41" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="C41" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D41" s="3"/>
+      <c r="C41" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D41" s="11"/>
     </row>
     <row r="42" ht="14.25">
-      <c r="A42" s="4">
+      <c r="A42" s="8">
         <v>11</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B42" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="C42" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D42" s="3" t="s">
+      <c r="C42" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D42" s="11" t="s">
         <v>214</v>
       </c>
     </row>
     <row r="43" ht="14.25">
-      <c r="A43" s="4"/>
-      <c r="B43" t="s">
+      <c r="A43" s="8"/>
+      <c r="B43" s="9" t="s">
         <v>215</v>
       </c>
-      <c r="C43" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D43" s="3"/>
+      <c r="C43" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D43" s="11"/>
     </row>
     <row r="44" ht="14.25">
-      <c r="A44" s="4"/>
-      <c r="B44" t="s">
+      <c r="A44" s="8"/>
+      <c r="B44" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="C44" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D44" s="3"/>
+      <c r="C44" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D44" s="11"/>
     </row>
     <row r="45" ht="14.25">
-      <c r="A45" s="4"/>
-      <c r="B45" t="s">
+      <c r="A45" s="8"/>
+      <c r="B45" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="C45" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D45" s="3"/>
+      <c r="C45" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D45" s="11"/>
     </row>
     <row r="46" ht="14.25">
-      <c r="A46" s="4">
+      <c r="A46" s="8">
         <v>12</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B46" s="9" t="s">
         <v>218</v>
       </c>
-      <c r="C46" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D46" s="3" t="s">
+      <c r="C46" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D46" s="11" t="s">
         <v>219</v>
       </c>
     </row>
     <row r="47" ht="14.25">
-      <c r="A47" s="4"/>
-      <c r="B47" t="s">
+      <c r="A47" s="8"/>
+      <c r="B47" s="9" t="s">
         <v>220</v>
       </c>
-      <c r="C47" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D47" s="3"/>
+      <c r="C47" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D47" s="11"/>
     </row>
     <row r="48" ht="14.25">
-      <c r="A48" s="4"/>
-      <c r="C48" s="1"/>
-      <c r="D48" s="3"/>
+      <c r="A48" s="8"/>
+      <c r="B48" s="9"/>
+      <c r="C48" s="10"/>
+      <c r="D48" s="11"/>
     </row>
     <row r="49" ht="14.25">
-      <c r="A49" s="4"/>
-      <c r="C49" s="1"/>
-      <c r="D49" s="3"/>
+      <c r="A49" s="8"/>
+      <c r="B49" s="9"/>
+      <c r="C49" s="10"/>
+      <c r="D49" s="11"/>
     </row>
     <row r="50" ht="14.25">
-      <c r="A50" s="4">
+      <c r="A50" s="8">
         <v>13</v>
       </c>
-      <c r="B50" t="s">
+      <c r="B50" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="C50" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D50" s="3" t="s">
+      <c r="C50" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D50" s="11" t="s">
         <v>222</v>
       </c>
     </row>
     <row r="51" ht="14.25">
-      <c r="A51" s="4"/>
-      <c r="B51" t="s">
+      <c r="A51" s="8"/>
+      <c r="B51" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="C51" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D51" s="3"/>
+      <c r="C51" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D51" s="11"/>
     </row>
     <row r="52" ht="14.25">
-      <c r="A52" s="4"/>
-      <c r="B52" t="s">
+      <c r="A52" s="8"/>
+      <c r="B52" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="C52" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D52" s="3"/>
+      <c r="C52" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D52" s="11"/>
     </row>
     <row r="53" ht="14.25">
-      <c r="A53" s="4"/>
-      <c r="B53" t="s">
+      <c r="A53" s="8"/>
+      <c r="B53" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="C53" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D53" s="3"/>
+      <c r="C53" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D53" s="11"/>
     </row>
     <row r="54" ht="14.25">
-      <c r="A54" s="4">
+      <c r="A54" s="8">
         <v>14</v>
       </c>
-      <c r="B54" t="s">
+      <c r="B54" s="9" t="s">
         <v>224</v>
       </c>
-      <c r="C54" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D54" s="3" t="s">
+      <c r="C54" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D54" s="11" t="s">
         <v>225</v>
       </c>
     </row>
     <row r="55" ht="14.25">
-      <c r="A55" s="4"/>
-      <c r="B55" t="s">
+      <c r="A55" s="8"/>
+      <c r="B55" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="C55" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D55" s="3"/>
+      <c r="C55" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D55" s="11"/>
     </row>
     <row r="56" ht="14.25">
-      <c r="A56" s="4"/>
-      <c r="B56" t="s">
+      <c r="A56" s="8"/>
+      <c r="B56" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="C56" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="D56" s="3"/>
+      <c r="C56" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="D56" s="11"/>
     </row>
     <row r="57" ht="14.25">
-      <c r="A57" s="4"/>
-      <c r="D57" s="3"/>
+      <c r="A57" s="8"/>
+      <c r="B57" s="9"/>
+      <c r="C57" s="10"/>
+      <c r="D57" s="11"/>
     </row>
     <row r="58" ht="14.25">
-      <c r="A58" s="4">
+      <c r="A58" s="8">
         <v>15</v>
       </c>
-      <c r="B58" t="s">
+      <c r="B58" s="9" t="s">
         <v>160</v>
       </c>
-      <c r="C58" s="9" t="s">
-        <v>137</v>
-      </c>
-      <c r="D58" s="10" t="s">
+      <c r="C58" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D58" s="11" t="s">
         <v>228</v>
       </c>
     </row>
     <row r="59" ht="14.25">
-      <c r="A59" s="4"/>
-      <c r="B59" t="s">
+      <c r="A59" s="8"/>
+      <c r="B59" s="9" t="s">
         <v>161</v>
       </c>
-      <c r="C59" s="9" t="s">
-        <v>137</v>
-      </c>
-      <c r="D59" s="3"/>
+      <c r="C59" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D59" s="11"/>
     </row>
     <row r="60" ht="14.25">
-      <c r="A60" s="4"/>
-      <c r="B60" t="s">
+      <c r="A60" s="8"/>
+      <c r="B60" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="C60" s="9" t="s">
-        <v>137</v>
-      </c>
-      <c r="D60" s="3"/>
+      <c r="C60" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D60" s="11"/>
     </row>
     <row r="61" ht="14.25">
-      <c r="A61" s="4"/>
-      <c r="B61" t="s">
+      <c r="A61" s="8"/>
+      <c r="B61" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="C61" s="9" t="s">
-        <v>137</v>
-      </c>
-      <c r="D61" s="3"/>
+      <c r="C61" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D61" s="11"/>
     </row>
     <row r="62" ht="14.25">
-      <c r="A62" s="4"/>
-      <c r="D62" s="3"/>
+      <c r="A62" s="8"/>
+      <c r="B62" s="9"/>
+      <c r="C62" s="10"/>
+      <c r="D62" s="11"/>
     </row>
     <row r="63" ht="14.25">
-      <c r="A63" s="4"/>
-      <c r="D63" s="3"/>
+      <c r="A63" s="8"/>
+      <c r="B63" s="9"/>
+      <c r="C63" s="10"/>
+      <c r="D63" s="11"/>
     </row>
     <row r="64" ht="14.25">
-      <c r="A64" s="4"/>
-      <c r="D64" s="3"/>
+      <c r="A64" s="8"/>
+      <c r="B64" s="9"/>
+      <c r="C64" s="10"/>
+      <c r="D64" s="11"/>
     </row>
     <row r="65" ht="14.25">
-      <c r="A65" s="4"/>
-      <c r="D65" s="3"/>
+      <c r="A65" s="8"/>
+      <c r="B65" s="9"/>
+      <c r="C65" s="10"/>
+      <c r="D65" s="11"/>
     </row>
     <row r="66" ht="14.25">
-      <c r="A66" s="4"/>
-      <c r="D66" s="3"/>
+      <c r="A66" s="8"/>
+      <c r="B66" s="9"/>
+      <c r="C66" s="10"/>
+      <c r="D66" s="11"/>
     </row>
     <row r="67" ht="14.25">
-      <c r="A67" s="4"/>
-      <c r="D67" s="3"/>
+      <c r="A67" s="8"/>
+      <c r="B67" s="9"/>
+      <c r="C67" s="10"/>
+      <c r="D67" s="11"/>
     </row>
     <row r="68" ht="14.25">
-      <c r="A68" s="4"/>
-      <c r="D68" s="3"/>
+      <c r="A68" s="8"/>
+      <c r="B68" s="9"/>
+      <c r="C68" s="10"/>
+      <c r="D68" s="11"/>
     </row>
     <row r="69" ht="14.25">
-      <c r="A69" s="4"/>
-      <c r="D69" s="3"/>
+      <c r="A69" s="8"/>
+      <c r="B69" s="9"/>
+      <c r="C69" s="10"/>
+      <c r="D69" s="11"/>
     </row>
     <row r="70" ht="14.25">
-      <c r="A70" s="4"/>
-      <c r="D70" s="3"/>
+      <c r="A70" s="8"/>
+      <c r="B70" s="9"/>
+      <c r="C70" s="10"/>
+      <c r="D70" s="11"/>
     </row>
     <row r="71" ht="14.25">
-      <c r="A71" s="4"/>
-      <c r="D71" s="3"/>
+      <c r="A71" s="8"/>
+      <c r="B71" s="9"/>
+      <c r="C71" s="10"/>
+      <c r="D71" s="11"/>
     </row>
     <row r="72" ht="14.25">
-      <c r="A72" s="4"/>
-      <c r="D72" s="3"/>
+      <c r="A72" s="8"/>
+      <c r="B72" s="9"/>
+      <c r="C72" s="10"/>
+      <c r="D72" s="11"/>
     </row>
     <row r="73" ht="14.25">
-      <c r="A73" s="4"/>
-      <c r="D73" s="3"/>
+      <c r="A73" s="8"/>
+      <c r="B73" s="9"/>
+      <c r="C73" s="10"/>
+      <c r="D73" s="11"/>
     </row>
     <row r="74" ht="14.25">
-      <c r="A74" s="4"/>
-      <c r="D74" s="3"/>
+      <c r="A74" s="8"/>
+      <c r="B74" s="9"/>
+      <c r="C74" s="10"/>
+      <c r="D74" s="11"/>
     </row>
     <row r="75" ht="14.25">
-      <c r="A75" s="4"/>
-      <c r="D75" s="3"/>
+      <c r="A75" s="8"/>
+      <c r="B75" s="9"/>
+      <c r="C75" s="10"/>
+      <c r="D75" s="11"/>
     </row>
     <row r="76" ht="14.25">
-      <c r="A76" s="4"/>
-      <c r="D76" s="3"/>
+      <c r="A76" s="8"/>
+      <c r="B76" s="9"/>
+      <c r="C76" s="10"/>
+      <c r="D76" s="11"/>
     </row>
     <row r="77" ht="14.25">
-      <c r="A77" s="4"/>
-      <c r="D77" s="3"/>
+      <c r="A77" s="8"/>
+      <c r="B77" s="9"/>
+      <c r="C77" s="10"/>
+      <c r="D77" s="11"/>
     </row>
     <row r="78" ht="14.25">
-      <c r="A78" s="4"/>
-      <c r="D78" s="3"/>
+      <c r="A78" s="8"/>
+      <c r="B78" s="9"/>
+      <c r="C78" s="10"/>
+      <c r="D78" s="11"/>
     </row>
     <row r="79" ht="14.25">
-      <c r="A79" s="4"/>
-      <c r="D79" s="3"/>
+      <c r="A79" s="8"/>
+      <c r="B79" s="9"/>
+      <c r="C79" s="10"/>
+      <c r="D79" s="11"/>
     </row>
     <row r="80" ht="14.25">
-      <c r="A80" s="4"/>
-      <c r="D80" s="3"/>
+      <c r="A80" s="8"/>
+      <c r="B80" s="9"/>
+      <c r="C80" s="10"/>
+      <c r="D80" s="11"/>
     </row>
     <row r="81" ht="14.25">
-      <c r="A81" s="4"/>
-      <c r="D81" s="3"/>
+      <c r="A81" s="8"/>
+      <c r="B81" s="9"/>
+      <c r="C81" s="10"/>
+      <c r="D81" s="11"/>
     </row>
     <row r="82" ht="14.25">
-      <c r="A82" s="4"/>
-      <c r="D82" s="3"/>
+      <c r="A82" s="8"/>
+      <c r="B82" s="9"/>
+      <c r="C82" s="10"/>
+      <c r="D82" s="11"/>
     </row>
     <row r="83" ht="14.25">
-      <c r="A83" s="4"/>
-      <c r="D83" s="3"/>
+      <c r="A83" s="8"/>
+      <c r="B83" s="9"/>
+      <c r="C83" s="10"/>
+      <c r="D83" s="11"/>
     </row>
     <row r="84" ht="14.25">
-      <c r="A84" s="4"/>
-      <c r="D84" s="3"/>
+      <c r="A84" s="8"/>
+      <c r="B84" s="9"/>
+      <c r="C84" s="10"/>
+      <c r="D84" s="11"/>
     </row>
     <row r="85" ht="14.25">
-      <c r="A85" s="4"/>
-      <c r="D85" s="3"/>
+      <c r="A85" s="8"/>
+      <c r="B85" s="9"/>
+      <c r="C85" s="10"/>
+      <c r="D85" s="11"/>
     </row>
     <row r="86" ht="14.25">
-      <c r="A86" s="4"/>
-      <c r="D86" s="3"/>
+      <c r="A86" s="8"/>
+      <c r="B86" s="9"/>
+      <c r="C86" s="10"/>
+      <c r="D86" s="11"/>
     </row>
     <row r="87" ht="14.25">
-      <c r="A87" s="4"/>
-      <c r="D87" s="3"/>
+      <c r="A87" s="8"/>
+      <c r="B87" s="9"/>
+      <c r="C87" s="10"/>
+      <c r="D87" s="11"/>
     </row>
     <row r="88" ht="14.25">
-      <c r="A88" s="4"/>
-      <c r="D88" s="3"/>
+      <c r="A88" s="8"/>
+      <c r="B88" s="9"/>
+      <c r="C88" s="10"/>
+      <c r="D88" s="11"/>
     </row>
     <row r="89" ht="14.25">
-      <c r="A89" s="4"/>
-      <c r="D89" s="3"/>
+      <c r="A89" s="8"/>
+      <c r="B89" s="9"/>
+      <c r="C89" s="10"/>
+      <c r="D89" s="11"/>
     </row>
     <row r="90" ht="14.25">
-      <c r="A90" s="4"/>
-      <c r="D90" s="3"/>
+      <c r="A90" s="8"/>
+      <c r="B90" s="9"/>
+      <c r="C90" s="10"/>
+      <c r="D90" s="11"/>
     </row>
     <row r="91" ht="14.25">
-      <c r="A91" s="4"/>
-      <c r="D91" s="3"/>
+      <c r="A91" s="8"/>
+      <c r="B91" s="9"/>
+      <c r="C91" s="10"/>
+      <c r="D91" s="11"/>
     </row>
     <row r="92" ht="14.25">
-      <c r="A92" s="4"/>
-      <c r="D92" s="3"/>
+      <c r="A92" s="8"/>
+      <c r="B92" s="9"/>
+      <c r="C92" s="10"/>
+      <c r="D92" s="11"/>
     </row>
     <row r="93" ht="14.25">
-      <c r="A93" s="4"/>
-      <c r="D93" s="3"/>
+      <c r="A93" s="8"/>
+      <c r="B93" s="9"/>
+      <c r="C93" s="10"/>
+      <c r="D93" s="11"/>
     </row>
     <row r="94" ht="14.25">
-      <c r="A94" s="4"/>
-      <c r="D94" s="3"/>
+      <c r="A94" s="8"/>
+      <c r="B94" s="9"/>
+      <c r="C94" s="10"/>
+      <c r="D94" s="11"/>
     </row>
     <row r="95" ht="14.25">
-      <c r="A95" s="4"/>
-      <c r="D95" s="3"/>
+      <c r="A95" s="8"/>
+      <c r="B95" s="9"/>
+      <c r="C95" s="10"/>
+      <c r="D95" s="11"/>
     </row>
     <row r="96" ht="14.25">
-      <c r="A96" s="4"/>
-      <c r="D96" s="3"/>
+      <c r="A96" s="8"/>
+      <c r="B96" s="9"/>
+      <c r="C96" s="10"/>
+      <c r="D96" s="11"/>
     </row>
     <row r="97" ht="14.25">
-      <c r="A97" s="4"/>
-      <c r="D97" s="3"/>
+      <c r="A97" s="8"/>
+      <c r="B97" s="9"/>
+      <c r="C97" s="10"/>
+      <c r="D97" s="11"/>
     </row>
     <row r="98" ht="14.25">
-      <c r="A98" s="4"/>
-      <c r="D98" s="3"/>
+      <c r="A98" s="8"/>
+      <c r="B98" s="9"/>
+      <c r="C98" s="10"/>
+      <c r="D98" s="11"/>
     </row>
     <row r="99" ht="14.25">
-      <c r="A99" s="4"/>
-      <c r="D99" s="3"/>
+      <c r="A99" s="8"/>
+      <c r="B99" s="9"/>
+      <c r="C99" s="10"/>
+      <c r="D99" s="11"/>
     </row>
     <row r="100" ht="14.25">
-      <c r="A100" s="4"/>
-      <c r="D100" s="3"/>
+      <c r="A100" s="8"/>
+      <c r="B100" s="9"/>
+      <c r="C100" s="10"/>
+      <c r="D100" s="11"/>
     </row>
     <row r="101" ht="14.25">
-      <c r="A101" s="4"/>
-      <c r="D101" s="3"/>
+      <c r="A101" s="8"/>
+      <c r="B101" s="9"/>
+      <c r="C101" s="10"/>
+      <c r="D101" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="50">
@@ -4066,9 +4168,9 @@
     <mergeCell ref="A98:A101"/>
     <mergeCell ref="D98:D101"/>
   </mergeCells>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <printOptions headings="0" gridLines="0" horizontalCentered="0" verticalCentered="0"/>
+  <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="1" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
   <headerFooter/>
 </worksheet>
 </file>
</xml_diff>